<commit_message>
fix: corregir consecutivo SOL-00054 para REQ-23718, asunto con SOL primero y seguimiento configurable a 3 dias y 1 semana para PO
</commit_message>
<xml_diff>
--- a/data/BD_Requisiciones.xlsx
+++ b/data/BD_Requisiciones.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y54"/>
+  <dimension ref="A1:Y55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -593,20 +593,16 @@
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K2" t="n">
+        <v>0</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M2" t="n">
+        <v>0</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -618,10 +614,8 @@
           <t>2026-02-12</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P2" t="n">
+        <v>0</v>
       </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
@@ -712,27 +706,21 @@
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K3" t="n">
+        <v>0</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M3" t="n">
+        <v>0</v>
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P3" t="n">
+        <v>0</v>
       </c>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
@@ -811,20 +799,16 @@
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K4" t="n">
+        <v>0</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M4" t="n">
+        <v>0</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -836,10 +820,8 @@
           <t>2026-03-02</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P4" t="n">
+        <v>0</v>
       </c>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
@@ -930,20 +912,16 @@
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K5" t="n">
+        <v>0</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M5" t="n">
+        <v>0</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -955,10 +933,8 @@
           <t>2026-03-02</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P5" t="n">
+        <v>0</v>
       </c>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
@@ -1049,20 +1025,16 @@
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K6" t="n">
+        <v>0</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M6" t="n">
+        <v>0</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -1074,10 +1046,8 @@
           <t>2026-03-02</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P6" t="n">
+        <v>0</v>
       </c>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
@@ -1168,20 +1138,16 @@
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K7" t="n">
+        <v>0</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M7" t="n">
+        <v>0</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -1193,10 +1159,8 @@
           <t>2026-03-02</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P7" t="n">
+        <v>0</v>
       </c>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
@@ -1300,27 +1264,21 @@
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K8" t="n">
+        <v>0</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M8" t="n">
+        <v>0</v>
       </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P8" t="n">
+        <v>0</v>
       </c>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
@@ -1399,20 +1357,16 @@
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K9" t="n">
+        <v>0</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M9" t="n">
+        <v>0</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -1424,10 +1378,8 @@
           <t>2026-03-06</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P9" t="n">
+        <v>0</v>
       </c>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
@@ -1522,27 +1474,21 @@
           <t>Multitarima Industrial</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>12500</t>
-        </is>
+      <c r="K10" t="n">
+        <v>12500</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="M10" t="n">
+        <v>1</v>
       </c>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P10" t="n">
+        <v>0</v>
       </c>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
@@ -1621,20 +1567,16 @@
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K11" t="n">
+        <v>0</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M11" t="n">
+        <v>0</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -1646,10 +1588,8 @@
           <t>2026-03-10</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P11" t="n">
+        <v>0</v>
       </c>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
@@ -1740,20 +1680,16 @@
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K12" t="n">
+        <v>0</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M12" t="n">
+        <v>0</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
@@ -1765,10 +1701,8 @@
           <t>2026-03-10</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P12" t="n">
+        <v>0</v>
       </c>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
@@ -1872,20 +1806,16 @@
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K13" t="n">
+        <v>0</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M13" t="n">
+        <v>0</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -1897,10 +1827,8 @@
           <t>2026-03-11</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P13" t="n">
+        <v>0</v>
       </c>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
@@ -1991,20 +1919,16 @@
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K14" t="n">
+        <v>0</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M14" t="n">
+        <v>0</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -2016,10 +1940,8 @@
           <t>2026-03-11</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P14" t="n">
+        <v>0</v>
       </c>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
@@ -2110,20 +2032,16 @@
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K15" t="n">
+        <v>0</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M15" t="n">
+        <v>0</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -2135,10 +2053,8 @@
           <t>2026-03-11</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P15" t="n">
+        <v>0</v>
       </c>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
@@ -2229,20 +2145,16 @@
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K16" t="n">
+        <v>0</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M16" t="n">
+        <v>0</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -2254,10 +2166,8 @@
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P16" t="n">
+        <v>0</v>
       </c>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
@@ -2348,20 +2258,16 @@
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K17" t="n">
+        <v>0</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M17" t="n">
+        <v>0</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
@@ -2373,10 +2279,8 @@
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P17" t="n">
+        <v>0</v>
       </c>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
@@ -2467,20 +2371,16 @@
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K18" t="n">
+        <v>0</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M18" t="n">
+        <v>0</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
@@ -2492,10 +2392,8 @@
           <t>2026-03-19</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P18" t="n">
+        <v>0</v>
       </c>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
@@ -2586,20 +2484,16 @@
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K19" t="n">
+        <v>0</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M19" t="n">
+        <v>0</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -2611,10 +2505,8 @@
           <t>2026-03-23</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P19" t="n">
+        <v>0</v>
       </c>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
@@ -2705,27 +2597,21 @@
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K20" t="n">
+        <v>0</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M20" t="n">
+        <v>0</v>
       </c>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P20" t="n">
+        <v>0</v>
       </c>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr"/>
@@ -2813,20 +2699,16 @@
           <t>Extractores Industriales</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>12500</t>
-        </is>
+      <c r="K21" t="n">
+        <v>12500</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="M21" t="n">
+        <v>3</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -2838,10 +2720,8 @@
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P21" t="n">
+        <v>0</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2936,20 +2816,16 @@
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K22" t="n">
+        <v>0</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M22" t="n">
+        <v>0</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
@@ -2961,10 +2837,8 @@
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P22" t="n">
+        <v>0</v>
       </c>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
@@ -3055,20 +2929,16 @@
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K23" t="n">
+        <v>0</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M23" t="n">
+        <v>0</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
@@ -3080,10 +2950,8 @@
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P23" t="n">
+        <v>0</v>
       </c>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
@@ -3174,27 +3042,21 @@
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K24" t="n">
+        <v>0</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M24" t="n">
+        <v>0</v>
       </c>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P24" t="n">
+        <v>0</v>
       </c>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
@@ -3273,20 +3135,16 @@
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K25" t="n">
+        <v>0</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M25" t="n">
+        <v>0</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
@@ -3298,10 +3156,8 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P25" t="n">
+        <v>0</v>
       </c>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
@@ -3392,20 +3248,16 @@
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K26" t="n">
+        <v>0</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M26" t="n">
+        <v>0</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
@@ -3417,10 +3269,8 @@
           <t>2026-03-31</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P26" t="n">
+        <v>0</v>
       </c>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
@@ -3511,20 +3361,16 @@
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K27" t="n">
+        <v>0</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M27" t="n">
+        <v>0</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
@@ -3536,10 +3382,8 @@
           <t>2026-03-31</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P27" t="n">
+        <v>0</v>
       </c>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
@@ -3630,20 +3474,16 @@
         </is>
       </c>
       <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K28" t="n">
+        <v>0</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M28" t="n">
+        <v>0</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
@@ -3655,10 +3495,8 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P28" t="n">
+        <v>0</v>
       </c>
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
@@ -3749,27 +3587,21 @@
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K29" t="n">
+        <v>0</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M29" t="n">
+        <v>0</v>
       </c>
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P29" t="n">
+        <v>0</v>
       </c>
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr"/>
@@ -3848,27 +3680,21 @@
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K30" t="n">
+        <v>0</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M30" t="n">
+        <v>0</v>
       </c>
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P30" t="n">
+        <v>0</v>
       </c>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
@@ -3947,27 +3773,21 @@
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K31" t="n">
+        <v>0</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M31" t="n">
+        <v>0</v>
       </c>
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P31" t="n">
+        <v>0</v>
       </c>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
@@ -4046,20 +3866,16 @@
         </is>
       </c>
       <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K32" t="n">
+        <v>0</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M32" t="n">
+        <v>0</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
@@ -4071,10 +3887,8 @@
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P32" t="n">
+        <v>0</v>
       </c>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
@@ -4168,20 +3982,16 @@
         </is>
       </c>
       <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K33" t="n">
+        <v>0</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M33" t="n">
+        <v>0</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
@@ -4193,10 +4003,8 @@
           <t>2026-04-10</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P33" t="n">
+        <v>0</v>
       </c>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
@@ -4287,20 +4095,16 @@
         </is>
       </c>
       <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K34" t="n">
+        <v>0</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M34" t="n">
+        <v>0</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
@@ -4312,10 +4116,8 @@
           <t>2026-04-10</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P34" t="n">
+        <v>0</v>
       </c>
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr">
@@ -4406,20 +4208,16 @@
         </is>
       </c>
       <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K35" t="n">
+        <v>0</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M35" t="n">
+        <v>0</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
@@ -4431,10 +4229,8 @@
           <t>2026-04-21</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P35" t="n">
+        <v>0</v>
       </c>
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr">
@@ -4525,27 +4321,21 @@
         </is>
       </c>
       <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K36" t="n">
+        <v>0</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M36" t="n">
+        <v>0</v>
       </c>
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P36" t="n">
+        <v>0</v>
       </c>
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr"/>
@@ -4624,27 +4414,21 @@
         </is>
       </c>
       <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K37" t="n">
+        <v>0</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M37" t="n">
+        <v>0</v>
       </c>
       <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P37" t="n">
+        <v>0</v>
       </c>
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr"/>
@@ -4723,27 +4507,21 @@
         </is>
       </c>
       <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K38" t="n">
+        <v>0</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M38" t="n">
+        <v>0</v>
       </c>
       <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P38" t="n">
+        <v>0</v>
       </c>
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr"/>
@@ -4822,27 +4600,21 @@
         </is>
       </c>
       <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K39" t="n">
+        <v>0</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M39" t="n">
+        <v>0</v>
       </c>
       <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P39" t="n">
+        <v>0</v>
       </c>
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr"/>
@@ -4925,27 +4697,21 @@
           <t>Maquinados y Troqueles</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>12500</t>
-        </is>
+      <c r="K40" t="n">
+        <v>12500</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="M40" t="n">
+        <v>2</v>
       </c>
       <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P40" t="n">
+        <v>0</v>
       </c>
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr"/>
@@ -5024,27 +4790,21 @@
         </is>
       </c>
       <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K41" t="n">
+        <v>0</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M41" t="n">
+        <v>0</v>
       </c>
       <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P41" t="n">
+        <v>0</v>
       </c>
       <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr"/>
@@ -5123,27 +4883,21 @@
         </is>
       </c>
       <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K42" t="n">
+        <v>0</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M42" t="n">
+        <v>0</v>
       </c>
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P42" t="n">
+        <v>0</v>
       </c>
       <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr"/>
@@ -5222,27 +4976,21 @@
         </is>
       </c>
       <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K43" t="n">
+        <v>0</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M43" t="n">
+        <v>0</v>
       </c>
       <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P43" t="n">
+        <v>0</v>
       </c>
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr"/>
@@ -5321,27 +5069,21 @@
         </is>
       </c>
       <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K44" t="n">
+        <v>0</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M44" t="n">
+        <v>0</v>
       </c>
       <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P44" t="n">
+        <v>0</v>
       </c>
       <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr"/>
@@ -5420,27 +5162,21 @@
         </is>
       </c>
       <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K45" t="n">
+        <v>0</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M45" t="n">
+        <v>0</v>
       </c>
       <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P45" t="n">
+        <v>0</v>
       </c>
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr"/>
@@ -5519,27 +5255,21 @@
         </is>
       </c>
       <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K46" t="n">
+        <v>0</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M46" t="n">
+        <v>0</v>
       </c>
       <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P46" t="n">
+        <v>0</v>
       </c>
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr"/>
@@ -5618,27 +5348,21 @@
         </is>
       </c>
       <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K47" t="n">
+        <v>0</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M47" t="n">
+        <v>0</v>
       </c>
       <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P47" t="n">
+        <v>0</v>
       </c>
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr"/>
@@ -5717,27 +5441,21 @@
         </is>
       </c>
       <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K48" t="n">
+        <v>0</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M48" t="n">
+        <v>0</v>
       </c>
       <c r="N48" t="inlineStr"/>
       <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P48" t="n">
+        <v>0</v>
       </c>
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr"/>
@@ -5816,27 +5534,21 @@
         </is>
       </c>
       <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K49" t="n">
+        <v>0</v>
       </c>
       <c r="L49" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M49" t="n">
+        <v>0</v>
       </c>
       <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P49" t="n">
+        <v>0</v>
       </c>
       <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr"/>
@@ -5919,27 +5631,21 @@
           <t>Equipos de Transporte y Lijado</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>12500</t>
-        </is>
+      <c r="K50" t="n">
+        <v>12500</v>
       </c>
       <c r="L50" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="M50" t="n">
+        <v>2</v>
       </c>
       <c r="N50" t="inlineStr"/>
       <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P50" t="n">
+        <v>0</v>
       </c>
       <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr"/>
@@ -6018,27 +5724,21 @@
         </is>
       </c>
       <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K51" t="n">
+        <v>0</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M51" t="n">
+        <v>0</v>
       </c>
       <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P51" t="n">
+        <v>0</v>
       </c>
       <c r="Q51" t="inlineStr"/>
       <c r="R51" t="inlineStr"/>
@@ -6117,20 +5817,16 @@
         </is>
       </c>
       <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K52" t="n">
+        <v>0</v>
       </c>
       <c r="L52" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M52" t="n">
+        <v>0</v>
       </c>
       <c r="N52" t="inlineStr">
         <is>
@@ -6142,10 +5838,8 @@
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="P52" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P52" t="n">
+        <v>0</v>
       </c>
       <c r="Q52" t="inlineStr"/>
       <c r="R52" t="inlineStr">
@@ -6236,20 +5930,16 @@
         </is>
       </c>
       <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K53" t="n">
+        <v>0</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="M53" t="n">
+        <v>0</v>
       </c>
       <c r="N53" t="inlineStr">
         <is>
@@ -6261,10 +5951,8 @@
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="P53" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P53" t="n">
+        <v>0</v>
       </c>
       <c r="Q53" t="inlineStr"/>
       <c r="R53" t="inlineStr">
@@ -6362,27 +6050,21 @@
           <t>COATEK Pintura</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>12500</t>
-        </is>
+      <c r="K54" t="n">
+        <v>12500</v>
       </c>
       <c r="L54" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="M54" t="n">
+        <v>1</v>
       </c>
       <c r="N54" t="inlineStr"/>
       <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P54" t="n">
+        <v>0</v>
       </c>
       <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr"/>
@@ -6411,6 +6093,97 @@
       <c r="Y54" t="inlineStr">
         <is>
           <t>2026-09-21 09:11:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>REQ-23718</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>SOL-00054</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Ing. Jesús Alberto Morales</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Materiales</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Refacciones Generales para maquinas Las</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Lentes pro superiores/inferiores, anillos cerámicos y boquillas D32 para cabezal de máquina de corte láser.</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>En Espera de Cotización</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="M55" t="n">
+        <v>0</v>
+      </c>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr"/>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>requisicion_REQ-23718.pdf</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>Autorizacion_SOL-00054_REQ-23718.eml</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr"/>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>Registrado formalmente en sistema. Consecutivo SOL-00054 asignado a Planta Metales.</t>
+        </is>
+      </c>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>2026-09-21 12:00:00</t>
+        </is>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>2026-09-21 12:25:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: integrar REQ-23718 (SOL-00054) y REQ-23775 (SOL-00055) con politicas estrictas para prevenir duplicados de requisicion
</commit_message>
<xml_diff>
--- a/data/BD_Requisiciones.xlsx
+++ b/data/BD_Requisiciones.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y55"/>
+  <dimension ref="A1:Y56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Ing. Jesús Alberto Morales</t>
+          <t>Bryan Alejandro Flores Mancinas</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -6129,7 +6129,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Lentes pro superiores/inferiores, anillos cerámicos y boquillas D32 para cabezal de máquina de corte láser.</t>
+          <t>Actualizado sin duplicar.</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -6146,36 +6146,22 @@
       <c r="K55" t="n">
         <v>0</v>
       </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>MXN</t>
-        </is>
-      </c>
+      <c r="L55" t="inlineStr"/>
       <c r="M55" t="n">
         <v>0</v>
       </c>
       <c r="N55" t="inlineStr"/>
       <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr"/>
+      <c r="P55" t="n">
+        <v>0</v>
+      </c>
       <c r="Q55" t="inlineStr"/>
       <c r="R55" t="inlineStr"/>
       <c r="S55" t="inlineStr"/>
-      <c r="T55" t="inlineStr">
-        <is>
-          <t>requisicion_REQ-23718.pdf</t>
-        </is>
-      </c>
-      <c r="U55" t="inlineStr">
-        <is>
-          <t>Autorizacion_SOL-00054_REQ-23718.eml</t>
-        </is>
-      </c>
+      <c r="T55" t="inlineStr"/>
+      <c r="U55" t="inlineStr"/>
       <c r="V55" t="inlineStr"/>
-      <c r="W55" t="inlineStr">
-        <is>
-          <t>Registrado formalmente en sistema. Consecutivo SOL-00054 asignado a Planta Metales.</t>
-        </is>
-      </c>
+      <c r="W55" t="inlineStr"/>
       <c r="X55" t="inlineStr">
         <is>
           <t>2026-09-21 12:00:00</t>
@@ -6183,7 +6169,100 @@
       </c>
       <c r="Y55" t="inlineStr">
         <is>
-          <t>2026-09-21 12:25:19</t>
+          <t>2026-09-21 12:44:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>REQ-23775</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>SOL-00055</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Bryan Alejandro Flores Mancinas</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Materiales</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Refacciones Generales para maquinas Las</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Consumibles y refacciones para cabezal láser: Lentes superiores/inferiores, anillos cerámicos y boquillas D32 (1.5 a 4.0). Fecha de entrega: 21/09/2026. Solicitado por Bryan Flores y autorizado por Ing. Jesús Morales.</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>En Espera de Cotización</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="M56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
+      <c r="P56" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="inlineStr"/>
+      <c r="S56" t="inlineStr"/>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>requisicion_REQ-23775.pdf</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>Autorizacion_SOL-00055_REQ-23775.eml</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr"/>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>Registrado formalmente en sistema. Consecutivo SOL-00055 asignado a Planta Metales.</t>
+        </is>
+      </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>2026-09-21 12:35:00</t>
+        </is>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>2026-09-21 12:40:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: actualización de data/BD_Requisiciones.xlsx desde Streamlit Cloud
</commit_message>
<xml_diff>
--- a/data/BD_Requisiciones.xlsx
+++ b/data/BD_Requisiciones.xlsx
@@ -6024,7 +6024,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>DEL LOCAL</t>
+          <t>Servicio de Mantenimieto de Máquina Coatek</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -6092,7 +6092,7 @@
       </c>
       <c r="Y54" t="inlineStr">
         <is>
-          <t>2026-09-21 16:47:42</t>
+          <t>2026-09-22 14:28:51</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(kanban): estilo Post-it con color de fondo completo, boton unico de apertura y selector en modal
</commit_message>
<xml_diff>
--- a/data/BD_Requisiciones.xlsx
+++ b/data/BD_Requisiciones.xlsx
@@ -663,7 +663,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -757,7 +761,11 @@
           <t>2026-09-22 16:37:42</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -871,7 +879,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -985,7 +997,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1099,7 +1115,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1213,7 +1233,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1320,7 +1344,11 @@
           <t>2026-09-22 16:37:48</t>
         </is>
       </c>
-      <c r="Z8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1434,7 +1462,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1532,7 +1564,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1646,7 +1682,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1760,7 +1800,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1887,7 +1931,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z13" t="inlineStr"/>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2001,7 +2049,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z14" t="inlineStr"/>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2115,7 +2167,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2229,7 +2285,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2343,7 +2403,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2457,7 +2521,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2571,7 +2639,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2665,7 +2737,11 @@
           <t>2026-09-22 16:55:19</t>
         </is>
       </c>
-      <c r="Z20" t="inlineStr"/>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2792,7 +2868,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z21" t="inlineStr"/>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2906,7 +2986,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z22" t="inlineStr"/>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3020,7 +3104,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3114,7 +3202,11 @@
           <t>2026-09-22 16:55:47</t>
         </is>
       </c>
-      <c r="Z24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3228,7 +3320,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3342,7 +3438,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3456,7 +3556,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3570,7 +3674,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3664,7 +3772,11 @@
           <t>2026-09-22 16:55:54</t>
         </is>
       </c>
-      <c r="Z29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3758,7 +3870,11 @@
           <t>2026-09-22 16:56:23</t>
         </is>
       </c>
-      <c r="Z30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3852,7 +3968,11 @@
           <t>2026-09-22 16:57:56</t>
         </is>
       </c>
-      <c r="Z31" t="inlineStr"/>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3966,7 +4086,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4083,7 +4207,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z33" t="inlineStr"/>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4197,7 +4325,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z34" t="inlineStr"/>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4311,7 +4443,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z35" t="inlineStr"/>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4405,7 +4541,11 @@
           <t>2026-09-22 16:58:09</t>
         </is>
       </c>
-      <c r="Z36" t="inlineStr"/>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4594,12 +4734,12 @@
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>2026-09-22 17:38:02</t>
+          <t>2026-09-21 09:11:20</t>
         </is>
       </c>
       <c r="Z38" t="inlineStr">
         <is>
-          <t>azul</t>
+          <t>amarillo</t>
         </is>
       </c>
     </row>
@@ -4695,7 +4835,11 @@
           <t>2026-09-22 16:58:49</t>
         </is>
       </c>
-      <c r="Z39" t="inlineStr"/>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4793,7 +4937,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z40" t="inlineStr"/>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4887,7 +5035,11 @@
           <t>2026-09-22 16:58:52</t>
         </is>
       </c>
-      <c r="Z41" t="inlineStr"/>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4981,7 +5133,11 @@
           <t>2026-09-22 17:12:13</t>
         </is>
       </c>
-      <c r="Z42" t="inlineStr"/>
+      <c r="Z42" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5075,7 +5231,11 @@
           <t>2026-09-22 16:59:05</t>
         </is>
       </c>
-      <c r="Z43" t="inlineStr"/>
+      <c r="Z43" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5169,7 +5329,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z44" t="inlineStr"/>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5263,7 +5427,11 @@
           <t>2026-09-22 17:11:52</t>
         </is>
       </c>
-      <c r="Z45" t="inlineStr"/>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5357,7 +5525,11 @@
           <t>2026-09-22 17:00:24</t>
         </is>
       </c>
-      <c r="Z46" t="inlineStr"/>
+      <c r="Z46" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5451,7 +5623,11 @@
           <t>2026-09-22 16:59:47</t>
         </is>
       </c>
-      <c r="Z47" t="inlineStr"/>
+      <c r="Z47" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5545,7 +5721,11 @@
           <t>2026-09-22 17:11:43</t>
         </is>
       </c>
-      <c r="Z48" t="inlineStr"/>
+      <c r="Z48" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5639,7 +5819,11 @@
           <t>2026-09-22 17:12:00</t>
         </is>
       </c>
-      <c r="Z49" t="inlineStr"/>
+      <c r="Z49" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5737,7 +5921,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z50" t="inlineStr"/>
+      <c r="Z50" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5831,7 +6019,11 @@
           <t>2026-09-22 16:59:25</t>
         </is>
       </c>
-      <c r="Z51" t="inlineStr"/>
+      <c r="Z51" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5945,7 +6137,11 @@
           <t>2026-09-21 09:11:20</t>
         </is>
       </c>
-      <c r="Z52" t="inlineStr"/>
+      <c r="Z52" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6059,7 +6255,11 @@
           <t>2026-09-22 14:35:14</t>
         </is>
       </c>
-      <c r="Z53" t="inlineStr"/>
+      <c r="Z53" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -6160,7 +6360,11 @@
           <t>2026-09-22 14:43:36</t>
         </is>
       </c>
-      <c r="Z54" t="inlineStr"/>
+      <c r="Z54" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6238,7 +6442,11 @@
           <t>2026-09-22 16:56:43</t>
         </is>
       </c>
-      <c r="Z55" t="inlineStr"/>
+      <c r="Z55" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -6332,7 +6540,11 @@
           <t>2026-09-22 16:56:39</t>
         </is>
       </c>
-      <c r="Z56" t="inlineStr"/>
+      <c r="Z56" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>